<commit_message>
step9: clearance columns in cm; keep Test 106 (MAD gate, no condition drop)
- SPSS export: scale T1 clearance/takeoff/landing mm->cm (1/10) so the
  clearance_* columns match the figure and Summary (were in mm).
- Test 106: remove the whole-condition exclusion of W1_H1/W1_H3/W2_H3 for
  hip/knee/thigh; rely on the 3*MAD stride gate + robust median instead, so
  those conditions are populated for 106 rather than left blank. Test 109's
  genuinely-missing joint conditions (W2_H1/W2_H3) stay blank.
- Regenerated SPSS, Summary, Results.md, .mat, and figures.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Results/Group Analysis/GroupCrossing_YoungAdults_SPSS.xlsx
+++ b/Results/Group Analysis/GroupCrossing_YoungAdults_SPSS.xlsx
@@ -2786,112 +2786,112 @@
         <v>101</v>
       </c>
       <c r="B2" s="0">
-        <v>149.80000000000001</v>
+        <v>14.98</v>
       </c>
       <c r="C2" s="0">
-        <v>127.101</v>
+        <v>12.710000000000001</v>
       </c>
       <c r="D2" s="0">
-        <v>78.162000000000006</v>
+        <v>7.8159999999999998</v>
       </c>
       <c r="E2" s="0">
-        <v>133.76599999999999</v>
+        <v>13.377000000000001</v>
       </c>
       <c r="F2" s="0">
-        <v>123.491</v>
+        <v>12.349</v>
       </c>
       <c r="G2" s="0">
-        <v>145.542</v>
+        <v>14.554</v>
       </c>
       <c r="H2" s="0">
-        <v>135.322</v>
+        <v>13.532</v>
       </c>
       <c r="I2" s="0">
-        <v>116.411</v>
+        <v>11.641</v>
       </c>
       <c r="J2" s="0">
-        <v>147.54400000000001</v>
+        <v>14.754</v>
       </c>
       <c r="K2" s="0">
-        <v>129.97800000000001</v>
+        <v>12.997999999999999</v>
       </c>
       <c r="L2" s="0">
-        <v>84.867999999999995</v>
+        <v>8.4870000000000001</v>
       </c>
       <c r="M2" s="0">
-        <v>138.43700000000001</v>
+        <v>13.843999999999999</v>
       </c>
       <c r="N2" s="0">
-        <v>701.35599999999999</v>
+        <v>70.135999999999996</v>
       </c>
       <c r="O2" s="0">
-        <v>818.30499999999995</v>
+        <v>81.829999999999998</v>
       </c>
       <c r="P2" s="0">
-        <v>747.02999999999997</v>
+        <v>74.703000000000003</v>
       </c>
       <c r="Q2" s="0">
-        <v>831.25999999999999</v>
+        <v>83.126000000000005</v>
       </c>
       <c r="R2" s="0">
-        <v>855.83299999999997</v>
+        <v>85.582999999999998</v>
       </c>
       <c r="S2" s="0">
-        <v>740.93499999999995</v>
+        <v>74.093000000000004</v>
       </c>
       <c r="T2" s="0">
-        <v>124.35899999999999</v>
+        <v>12.436</v>
       </c>
       <c r="U2" s="0">
-        <v>451.98899999999998</v>
+        <v>45.198999999999998</v>
       </c>
       <c r="V2" s="0">
-        <v>153.95099999999999</v>
+        <v>15.395</v>
       </c>
       <c r="W2" s="0">
-        <v>131.55000000000001</v>
+        <v>13.154999999999999</v>
       </c>
       <c r="X2" s="0">
-        <v>156.43100000000001</v>
+        <v>15.643000000000001</v>
       </c>
       <c r="Y2" s="0">
-        <v>169.45699999999999</v>
+        <v>16.946000000000002</v>
       </c>
       <c r="Z2" s="0">
-        <v>296.55599999999998</v>
+        <v>29.655999999999999</v>
       </c>
       <c r="AA2" s="0">
-        <v>260.892</v>
+        <v>26.088999999999999</v>
       </c>
       <c r="AB2" s="0">
-        <v>263.435</v>
+        <v>26.343</v>
       </c>
       <c r="AC2" s="0">
-        <v>177.15100000000001</v>
+        <v>17.715</v>
       </c>
       <c r="AD2" s="0">
-        <v>213.06</v>
+        <v>21.306000000000001</v>
       </c>
       <c r="AE2" s="0">
-        <v>471.92599999999999</v>
+        <v>47.192999999999998</v>
       </c>
       <c r="AF2" s="0">
-        <v>1045.327</v>
+        <v>104.533</v>
       </c>
       <c r="AG2" s="0">
-        <v>1034.086</v>
+        <v>103.40900000000001</v>
       </c>
       <c r="AH2" s="0">
-        <v>1013.563</v>
+        <v>101.35599999999999</v>
       </c>
       <c r="AI2" s="0">
-        <v>949.67700000000002</v>
+        <v>94.968000000000004</v>
       </c>
       <c r="AJ2" s="0">
-        <v>741.34100000000001</v>
+        <v>74.134</v>
       </c>
       <c r="AK2" s="0">
-        <v>924.70399999999995</v>
+        <v>92.469999999999999</v>
       </c>
       <c r="AL2" s="0">
         <v>180.19900000000001</v>
@@ -3952,112 +3952,112 @@
         <v>102</v>
       </c>
       <c r="B3" s="0">
-        <v>257.31200000000001</v>
+        <v>25.731000000000002</v>
       </c>
       <c r="C3" s="0">
-        <v>259.14600000000002</v>
+        <v>25.914999999999999</v>
       </c>
       <c r="D3" s="0">
-        <v>282.78699999999998</v>
+        <v>28.279</v>
       </c>
       <c r="E3" s="0">
-        <v>241.85900000000001</v>
+        <v>24.186</v>
       </c>
       <c r="F3" s="0">
-        <v>277.49799999999999</v>
+        <v>27.75</v>
       </c>
       <c r="G3" s="0">
-        <v>249.697</v>
+        <v>24.969999999999999</v>
       </c>
       <c r="H3" s="0">
-        <v>165.29400000000001</v>
+        <v>16.529</v>
       </c>
       <c r="I3" s="0">
-        <v>154.762</v>
+        <v>15.476000000000001</v>
       </c>
       <c r="J3" s="0">
-        <v>105.063</v>
+        <v>10.506</v>
       </c>
       <c r="K3" s="0">
-        <v>201.857</v>
+        <v>20.186</v>
       </c>
       <c r="L3" s="0">
-        <v>113.852</v>
+        <v>11.385</v>
       </c>
       <c r="M3" s="0">
-        <v>93.292000000000002</v>
+        <v>9.3290000000000006</v>
       </c>
       <c r="N3" s="0">
-        <v>1045.6669999999999</v>
+        <v>104.56699999999999</v>
       </c>
       <c r="O3" s="0">
-        <v>1097.6859999999999</v>
+        <v>109.76900000000001</v>
       </c>
       <c r="P3" s="0">
-        <v>1085.075</v>
+        <v>108.50700000000001</v>
       </c>
       <c r="Q3" s="0">
-        <v>979.80999999999995</v>
+        <v>97.980999999999995</v>
       </c>
       <c r="R3" s="0">
-        <v>1067.8679999999999</v>
+        <v>106.78700000000001</v>
       </c>
       <c r="S3" s="0">
-        <v>1025.425</v>
+        <v>102.542</v>
       </c>
       <c r="T3" s="0">
-        <v>248.75299999999999</v>
+        <v>24.875</v>
       </c>
       <c r="U3" s="0">
-        <v>273.22399999999999</v>
+        <v>27.321999999999999</v>
       </c>
       <c r="V3" s="0">
-        <v>239.161</v>
+        <v>23.916</v>
       </c>
       <c r="W3" s="0">
-        <v>228.46799999999999</v>
+        <v>22.847000000000001</v>
       </c>
       <c r="X3" s="0">
-        <v>225.66499999999999</v>
+        <v>22.567</v>
       </c>
       <c r="Y3" s="0">
-        <v>209.15000000000001</v>
+        <v>20.914999999999999</v>
       </c>
       <c r="Z3" s="0">
-        <v>341.28699999999998</v>
+        <v>34.128999999999998</v>
       </c>
       <c r="AA3" s="0">
-        <v>298.50400000000002</v>
+        <v>29.850000000000001</v>
       </c>
       <c r="AB3" s="0">
-        <v>362.01900000000001</v>
+        <v>36.201999999999998</v>
       </c>
       <c r="AC3" s="0">
-        <v>249.28899999999999</v>
+        <v>24.928999999999998</v>
       </c>
       <c r="AD3" s="0">
-        <v>265.863</v>
+        <v>26.585999999999999</v>
       </c>
       <c r="AE3" s="0">
-        <v>282.983</v>
+        <v>28.297999999999998</v>
       </c>
       <c r="AF3" s="0">
-        <v>1093.002</v>
+        <v>109.3</v>
       </c>
       <c r="AG3" s="0">
-        <v>1116.2729999999999</v>
+        <v>111.627</v>
       </c>
       <c r="AH3" s="0">
-        <v>1155.825</v>
+        <v>115.583</v>
       </c>
       <c r="AI3" s="0">
-        <v>1021.275</v>
+        <v>102.128</v>
       </c>
       <c r="AJ3" s="0">
-        <v>1058.5740000000001</v>
+        <v>105.857</v>
       </c>
       <c r="AK3" s="0">
-        <v>1089.634</v>
+        <v>108.96299999999999</v>
       </c>
       <c r="AL3" s="0">
         <v>176.28999999999999</v>
@@ -5118,112 +5118,112 @@
         <v>103</v>
       </c>
       <c r="B4" s="0">
-        <v>219.31899999999999</v>
+        <v>21.931999999999999</v>
       </c>
       <c r="C4" s="0">
-        <v>180.86799999999999</v>
+        <v>18.087</v>
       </c>
       <c r="D4" s="0">
-        <v>211.34899999999999</v>
+        <v>21.135000000000002</v>
       </c>
       <c r="E4" s="0">
-        <v>228.85499999999999</v>
+        <v>22.885999999999999</v>
       </c>
       <c r="F4" s="0">
-        <v>189.44499999999999</v>
+        <v>18.943999999999999</v>
       </c>
       <c r="G4" s="0">
-        <v>163.33699999999999</v>
+        <v>16.334</v>
       </c>
       <c r="H4" s="0">
-        <v>215.33600000000001</v>
+        <v>21.533999999999999</v>
       </c>
       <c r="I4" s="0">
-        <v>202.94900000000001</v>
+        <v>20.295000000000002</v>
       </c>
       <c r="J4" s="0">
-        <v>206.233</v>
+        <v>20.623000000000001</v>
       </c>
       <c r="K4" s="0">
-        <v>219.32300000000001</v>
+        <v>21.931999999999999</v>
       </c>
       <c r="L4" s="0">
-        <v>239.923</v>
+        <v>23.992000000000001</v>
       </c>
       <c r="M4" s="0">
-        <v>202.351</v>
+        <v>20.234999999999999</v>
       </c>
       <c r="N4" s="0">
-        <v>1042.5340000000001</v>
+        <v>104.253</v>
       </c>
       <c r="O4" s="0">
-        <v>1090.9739999999999</v>
+        <v>109.09699999999999</v>
       </c>
       <c r="P4" s="0">
-        <v>1021.191</v>
+        <v>102.119</v>
       </c>
       <c r="Q4" s="0">
-        <v>1200.1389999999999</v>
+        <v>120.014</v>
       </c>
       <c r="R4" s="0">
-        <v>994.11000000000001</v>
+        <v>99.411000000000001</v>
       </c>
       <c r="S4" s="0">
-        <v>1145.5119999999999</v>
+        <v>114.551</v>
       </c>
       <c r="T4" s="0">
-        <v>261.67599999999999</v>
+        <v>26.167999999999999</v>
       </c>
       <c r="U4" s="0">
-        <v>304.64999999999998</v>
+        <v>30.465</v>
       </c>
       <c r="V4" s="0">
-        <v>230.53100000000001</v>
+        <v>23.053000000000001</v>
       </c>
       <c r="W4" s="0">
-        <v>306.26600000000002</v>
+        <v>30.626999999999999</v>
       </c>
       <c r="X4" s="0">
-        <v>210.84</v>
+        <v>21.084</v>
       </c>
       <c r="Y4" s="0">
-        <v>296.18599999999998</v>
+        <v>29.619</v>
       </c>
       <c r="Z4" s="0">
-        <v>241.678</v>
+        <v>24.167999999999999</v>
       </c>
       <c r="AA4" s="0">
-        <v>278.79199999999997</v>
+        <v>27.879000000000001</v>
       </c>
       <c r="AB4" s="0">
-        <v>289.072</v>
+        <v>28.907</v>
       </c>
       <c r="AC4" s="0">
-        <v>221.63800000000001</v>
+        <v>22.164000000000001</v>
       </c>
       <c r="AD4" s="0">
-        <v>263.94400000000002</v>
+        <v>26.393999999999998</v>
       </c>
       <c r="AE4" s="0">
-        <v>198.88399999999999</v>
+        <v>19.888000000000002</v>
       </c>
       <c r="AF4" s="0">
-        <v>1021.0119999999999</v>
+        <v>102.101</v>
       </c>
       <c r="AG4" s="0">
-        <v>1093.326</v>
+        <v>109.333</v>
       </c>
       <c r="AH4" s="0">
-        <v>1145.2380000000001</v>
+        <v>114.524</v>
       </c>
       <c r="AI4" s="0">
-        <v>1053.9590000000001</v>
+        <v>105.396</v>
       </c>
       <c r="AJ4" s="0">
-        <v>1095.03</v>
+        <v>109.503</v>
       </c>
       <c r="AK4" s="0">
-        <v>1037.2329999999999</v>
+        <v>103.723</v>
       </c>
       <c r="AL4" s="0">
         <v>164.751</v>
@@ -6284,112 +6284,112 @@
         <v>104</v>
       </c>
       <c r="B5" s="0">
-        <v>191.58500000000001</v>
+        <v>19.158999999999999</v>
       </c>
       <c r="C5" s="0">
-        <v>202.702</v>
+        <v>20.27</v>
       </c>
       <c r="D5" s="0">
-        <v>193.55799999999999</v>
+        <v>19.356000000000002</v>
       </c>
       <c r="E5" s="0">
-        <v>146.75200000000001</v>
+        <v>14.675000000000001</v>
       </c>
       <c r="F5" s="0">
-        <v>199.709</v>
+        <v>19.971</v>
       </c>
       <c r="G5" s="0">
-        <v>182.85300000000001</v>
+        <v>18.285</v>
       </c>
       <c r="H5" s="0">
-        <v>308.78500000000003</v>
+        <v>30.879000000000001</v>
       </c>
       <c r="I5" s="0">
-        <v>333.892</v>
+        <v>33.389000000000003</v>
       </c>
       <c r="J5" s="0">
-        <v>263.29000000000002</v>
+        <v>26.329000000000001</v>
       </c>
       <c r="K5" s="0">
-        <v>261.57900000000001</v>
+        <v>26.158000000000001</v>
       </c>
       <c r="L5" s="0">
-        <v>297.85700000000003</v>
+        <v>29.786000000000001</v>
       </c>
       <c r="M5" s="0">
-        <v>307.69299999999998</v>
+        <v>30.768999999999998</v>
       </c>
       <c r="N5" s="0">
-        <v>681.59299999999996</v>
+        <v>68.159000000000006</v>
       </c>
       <c r="O5" s="0">
-        <v>718.81100000000004</v>
+        <v>71.881</v>
       </c>
       <c r="P5" s="0">
-        <v>514.07600000000002</v>
+        <v>51.408000000000001</v>
       </c>
       <c r="Q5" s="0">
-        <v>707.40800000000002</v>
+        <v>70.741</v>
       </c>
       <c r="R5" s="0">
-        <v>589.03899999999999</v>
+        <v>58.904000000000003</v>
       </c>
       <c r="S5" s="0">
-        <v>655.34400000000005</v>
+        <v>65.534000000000006</v>
       </c>
       <c r="T5" s="0">
-        <v>183.87799999999999</v>
+        <v>18.388000000000002</v>
       </c>
       <c r="U5" s="0">
-        <v>150.98099999999999</v>
+        <v>15.098000000000001</v>
       </c>
       <c r="V5" s="0">
-        <v>145.06100000000001</v>
+        <v>14.506</v>
       </c>
       <c r="W5" s="0">
-        <v>155.14099999999999</v>
+        <v>15.513999999999999</v>
       </c>
       <c r="X5" s="0">
-        <v>135.19499999999999</v>
+        <v>13.519</v>
       </c>
       <c r="Y5" s="0">
-        <v>111.051</v>
+        <v>11.105</v>
       </c>
       <c r="Z5" s="0">
-        <v>519.00400000000002</v>
+        <v>51.899999999999999</v>
       </c>
       <c r="AA5" s="0">
-        <v>209.666</v>
+        <v>20.966999999999999</v>
       </c>
       <c r="AB5" s="0">
-        <v>170.41499999999999</v>
+        <v>17.042000000000002</v>
       </c>
       <c r="AC5" s="0">
-        <v>464.36599999999999</v>
+        <v>46.436999999999998</v>
       </c>
       <c r="AD5" s="0">
-        <v>140.62299999999999</v>
+        <v>14.061999999999999</v>
       </c>
       <c r="AE5" s="0">
-        <v>47.326000000000001</v>
+        <v>4.7329999999999997</v>
       </c>
       <c r="AF5" s="0">
-        <v>945.69399999999996</v>
+        <v>94.569000000000003</v>
       </c>
       <c r="AG5" s="0">
-        <v>736.26599999999996</v>
+        <v>73.626999999999995</v>
       </c>
       <c r="AH5" s="0">
-        <v>481.43299999999999</v>
+        <v>48.143000000000001</v>
       </c>
       <c r="AI5" s="0">
-        <v>924.92899999999997</v>
+        <v>92.492999999999995</v>
       </c>
       <c r="AJ5" s="0">
-        <v>448.88400000000001</v>
+        <v>44.887999999999998</v>
       </c>
       <c r="AK5" s="0">
-        <v>777.40700000000004</v>
+        <v>77.741</v>
       </c>
       <c r="AL5" s="0">
         <v>156.81999999999999</v>
@@ -7450,112 +7450,112 @@
         <v>105</v>
       </c>
       <c r="B6" s="0">
-        <v>144.20699999999999</v>
+        <v>14.420999999999999</v>
       </c>
       <c r="C6" s="0">
-        <v>156.529</v>
+        <v>15.653</v>
       </c>
       <c r="D6" s="0">
-        <v>108.252</v>
+        <v>10.824999999999999</v>
       </c>
       <c r="E6" s="0">
-        <v>152.416</v>
+        <v>15.242000000000001</v>
       </c>
       <c r="F6" s="0">
-        <v>130.334</v>
+        <v>13.032999999999999</v>
       </c>
       <c r="G6" s="0">
-        <v>116.70399999999999</v>
+        <v>11.67</v>
       </c>
       <c r="H6" s="0">
-        <v>83.417000000000002</v>
+        <v>8.3420000000000005</v>
       </c>
       <c r="I6" s="0">
-        <v>115.16800000000001</v>
+        <v>11.516999999999999</v>
       </c>
       <c r="J6" s="0">
-        <v>135.47200000000001</v>
+        <v>13.547000000000001</v>
       </c>
       <c r="K6" s="0">
-        <v>119.733</v>
+        <v>11.973000000000001</v>
       </c>
       <c r="L6" s="0">
-        <v>60.098999999999997</v>
+        <v>6.0099999999999998</v>
       </c>
       <c r="M6" s="0">
-        <v>119.20999999999999</v>
+        <v>11.920999999999999</v>
       </c>
       <c r="N6" s="0">
-        <v>723.77499999999998</v>
+        <v>72.376999999999995</v>
       </c>
       <c r="O6" s="0">
-        <v>746.27099999999996</v>
+        <v>74.626999999999995</v>
       </c>
       <c r="P6" s="0">
-        <v>682.30600000000004</v>
+        <v>68.230999999999995</v>
       </c>
       <c r="Q6" s="0">
-        <v>627.69600000000003</v>
+        <v>62.770000000000003</v>
       </c>
       <c r="R6" s="0">
-        <v>654.50699999999995</v>
+        <v>65.450999999999993</v>
       </c>
       <c r="S6" s="0">
-        <v>635.95799999999997</v>
+        <v>63.595999999999997</v>
       </c>
       <c r="T6" s="0">
-        <v>161.43799999999999</v>
+        <v>16.143999999999998</v>
       </c>
       <c r="U6" s="0">
-        <v>160.85400000000001</v>
+        <v>16.085000000000001</v>
       </c>
       <c r="V6" s="0">
-        <v>107.05</v>
+        <v>10.705</v>
       </c>
       <c r="W6" s="0">
-        <v>116.66800000000001</v>
+        <v>11.667</v>
       </c>
       <c r="X6" s="0">
-        <v>96.986000000000004</v>
+        <v>9.6989999999999998</v>
       </c>
       <c r="Y6" s="0">
-        <v>102.649</v>
+        <v>10.265000000000001</v>
       </c>
       <c r="Z6" s="0">
-        <v>346.971</v>
+        <v>34.697000000000003</v>
       </c>
       <c r="AA6" s="0">
-        <v>124.643</v>
+        <v>12.464</v>
       </c>
       <c r="AB6" s="0">
-        <v>178.52799999999999</v>
+        <v>17.853000000000002</v>
       </c>
       <c r="AC6" s="0">
-        <v>81.293999999999997</v>
+        <v>8.1289999999999996</v>
       </c>
       <c r="AD6" s="0">
-        <v>110.863</v>
+        <v>11.086</v>
       </c>
       <c r="AE6" s="0">
-        <v>110.557</v>
+        <v>11.055999999999999</v>
       </c>
       <c r="AF6" s="0">
-        <v>674.17600000000004</v>
+        <v>67.418000000000006</v>
       </c>
       <c r="AG6" s="0">
-        <v>634.17399999999998</v>
+        <v>63.417000000000002</v>
       </c>
       <c r="AH6" s="0">
-        <v>711.36400000000003</v>
+        <v>71.135999999999996</v>
       </c>
       <c r="AI6" s="0">
-        <v>568.74000000000001</v>
+        <v>56.874000000000002</v>
       </c>
       <c r="AJ6" s="0">
-        <v>623.55399999999997</v>
+        <v>62.354999999999997</v>
       </c>
       <c r="AK6" s="0">
-        <v>603.54100000000005</v>
+        <v>60.353999999999999</v>
       </c>
       <c r="AL6" s="0">
         <v>142.52799999999999</v>
@@ -8616,112 +8616,112 @@
         <v>106</v>
       </c>
       <c r="B7" s="0">
-        <v>155.27500000000001</v>
+        <v>15.528</v>
       </c>
       <c r="C7" s="0">
-        <v>192.18199999999999</v>
+        <v>19.218</v>
       </c>
       <c r="D7" s="0">
-        <v>118.169</v>
+        <v>11.817</v>
       </c>
       <c r="E7" s="0">
-        <v>99.162000000000006</v>
+        <v>9.9160000000000004</v>
       </c>
       <c r="F7" s="0">
-        <v>167.60900000000001</v>
+        <v>16.760999999999999</v>
       </c>
       <c r="G7" s="0">
-        <v>133.73099999999999</v>
+        <v>13.372999999999999</v>
       </c>
       <c r="H7" s="0">
-        <v>92.402000000000001</v>
+        <v>9.2400000000000002</v>
       </c>
       <c r="I7" s="0">
-        <v>136.90600000000001</v>
+        <v>13.691000000000001</v>
       </c>
       <c r="J7" s="0">
-        <v>58.338000000000001</v>
+        <v>5.8339999999999996</v>
       </c>
       <c r="K7" s="0">
-        <v>124.274</v>
+        <v>12.427</v>
       </c>
       <c r="L7" s="0">
-        <v>148.851</v>
+        <v>14.885</v>
       </c>
       <c r="M7" s="0">
-        <v>203.16900000000001</v>
+        <v>20.317</v>
       </c>
       <c r="N7" s="0">
-        <v>799.28999999999996</v>
+        <v>79.929000000000002</v>
       </c>
       <c r="O7" s="0">
-        <v>940.18100000000004</v>
+        <v>94.018000000000001</v>
       </c>
       <c r="P7" s="0">
-        <v>987.95600000000002</v>
+        <v>98.796000000000006</v>
       </c>
       <c r="Q7" s="0">
-        <v>1065.4960000000001</v>
+        <v>106.55</v>
       </c>
       <c r="R7" s="0">
-        <v>941.19500000000005</v>
+        <v>94.119</v>
       </c>
       <c r="S7" s="0">
-        <v>948.31500000000005</v>
+        <v>94.831000000000003</v>
       </c>
       <c r="T7" s="0">
-        <v>164.52500000000001</v>
+        <v>16.452999999999999</v>
       </c>
       <c r="U7" s="0">
-        <v>269.44900000000001</v>
+        <v>26.945</v>
       </c>
       <c r="V7" s="0">
-        <v>267.875</v>
+        <v>26.788</v>
       </c>
       <c r="W7" s="0">
-        <v>309.05900000000003</v>
+        <v>30.905999999999999</v>
       </c>
       <c r="X7" s="0">
-        <v>243.65199999999999</v>
+        <v>24.364999999999998</v>
       </c>
       <c r="Y7" s="0">
-        <v>206.71100000000001</v>
+        <v>20.670999999999999</v>
       </c>
       <c r="Z7" s="0">
-        <v>270.36799999999999</v>
+        <v>27.036999999999999</v>
       </c>
       <c r="AA7" s="0">
-        <v>206.078</v>
+        <v>20.608000000000001</v>
       </c>
       <c r="AB7" s="0">
-        <v>202.96600000000001</v>
+        <v>20.297000000000001</v>
       </c>
       <c r="AC7" s="0">
-        <v>147.96199999999999</v>
+        <v>14.795999999999999</v>
       </c>
       <c r="AD7" s="0">
-        <v>154.386</v>
+        <v>15.439</v>
       </c>
       <c r="AE7" s="0">
-        <v>192.215</v>
+        <v>19.222000000000001</v>
       </c>
       <c r="AF7" s="0">
-        <v>974.87199999999996</v>
+        <v>97.486999999999995</v>
       </c>
       <c r="AG7" s="0">
-        <v>893.62800000000004</v>
+        <v>89.363</v>
       </c>
       <c r="AH7" s="0">
-        <v>930.05399999999997</v>
+        <v>93.004999999999995</v>
       </c>
       <c r="AI7" s="0">
-        <v>881.76499999999999</v>
+        <v>88.177000000000007</v>
       </c>
       <c r="AJ7" s="0">
-        <v>850.86900000000003</v>
+        <v>85.087000000000003</v>
       </c>
       <c r="AK7" s="0">
-        <v>867.27099999999996</v>
+        <v>86.727000000000004</v>
       </c>
       <c r="AL7" s="0">
         <v>141.18199999999999</v>
@@ -8879,57 +8879,81 @@
       <c r="CK7" s="0">
         <v>46.844000000000001</v>
       </c>
-      <c r="CL7" s="0"/>
+      <c r="CL7" s="0">
+        <v>29.968</v>
+      </c>
       <c r="CM7" s="0">
         <v>75.823999999999998</v>
       </c>
-      <c r="CN7" s="0"/>
+      <c r="CN7" s="0">
+        <v>36.895000000000003</v>
+      </c>
       <c r="CO7" s="0">
         <v>37.932000000000002</v>
       </c>
       <c r="CP7" s="0">
         <v>42.509</v>
       </c>
-      <c r="CQ7" s="0"/>
-      <c r="CR7" s="0"/>
+      <c r="CQ7" s="0">
+        <v>60.479999999999997</v>
+      </c>
+      <c r="CR7" s="0">
+        <v>23.052</v>
+      </c>
       <c r="CS7" s="0">
         <v>36.811999999999998</v>
       </c>
-      <c r="CT7" s="0"/>
+      <c r="CT7" s="0">
+        <v>42.279000000000003</v>
+      </c>
       <c r="CU7" s="0">
         <v>32.301000000000002</v>
       </c>
       <c r="CV7" s="0">
         <v>20.425999999999998</v>
       </c>
-      <c r="CW7" s="0"/>
+      <c r="CW7" s="0">
+        <v>28.919</v>
+      </c>
       <c r="CX7" s="0">
         <v>16.748000000000001</v>
       </c>
-      <c r="CY7" s="0"/>
+      <c r="CY7" s="0">
+        <v>57.133000000000003</v>
+      </c>
       <c r="CZ7" s="0">
         <v>87.706000000000003</v>
       </c>
-      <c r="DA7" s="0"/>
+      <c r="DA7" s="0">
+        <v>93.936000000000007</v>
+      </c>
       <c r="DB7" s="0">
         <v>43.975999999999999</v>
       </c>
       <c r="DC7" s="0">
         <v>86.609999999999999</v>
       </c>
-      <c r="DD7" s="0"/>
-      <c r="DE7" s="0"/>
+      <c r="DD7" s="0">
+        <v>66.489999999999995</v>
+      </c>
+      <c r="DE7" s="0">
+        <v>17.943000000000001</v>
+      </c>
       <c r="DF7" s="0">
         <v>27.395</v>
       </c>
-      <c r="DG7" s="0"/>
+      <c r="DG7" s="0">
+        <v>33.232999999999997</v>
+      </c>
       <c r="DH7" s="0">
         <v>93.325000000000003</v>
       </c>
       <c r="DI7" s="0">
         <v>30.792999999999999</v>
       </c>
-      <c r="DJ7" s="0"/>
+      <c r="DJ7" s="0">
+        <v>106.02</v>
+      </c>
       <c r="DK7" s="0">
         <v>57.911999999999999</v>
       </c>
@@ -8972,57 +8996,81 @@
       <c r="DX7" s="0">
         <v>8.2319999999999993</v>
       </c>
-      <c r="DY7" s="0"/>
+      <c r="DY7" s="0">
+        <v>-13.789999999999999</v>
+      </c>
       <c r="DZ7" s="0">
         <v>-15.231999999999999</v>
       </c>
-      <c r="EA7" s="0"/>
+      <c r="EA7" s="0">
+        <v>-15.377000000000001</v>
+      </c>
       <c r="EB7" s="0">
         <v>-11.234999999999999</v>
       </c>
       <c r="EC7" s="0">
         <v>-21.981000000000002</v>
       </c>
-      <c r="ED7" s="0"/>
-      <c r="EE7" s="0"/>
+      <c r="ED7" s="0">
+        <v>-7.6210000000000004</v>
+      </c>
+      <c r="EE7" s="0">
+        <v>-2.6549999999999998</v>
+      </c>
       <c r="EF7" s="0">
         <v>-8.8520000000000003</v>
       </c>
-      <c r="EG7" s="0"/>
+      <c r="EG7" s="0">
+        <v>-8.4700000000000006</v>
+      </c>
       <c r="EH7" s="0">
         <v>-22.593</v>
       </c>
       <c r="EI7" s="0">
         <v>-14.754</v>
       </c>
-      <c r="EJ7" s="0"/>
+      <c r="EJ7" s="0">
+        <v>-17.393000000000001</v>
+      </c>
       <c r="EK7" s="0">
         <v>-3.431</v>
       </c>
-      <c r="EL7" s="0"/>
+      <c r="EL7" s="0">
+        <v>-3.1419999999999999</v>
+      </c>
       <c r="EM7" s="0">
         <v>-3.79</v>
       </c>
-      <c r="EN7" s="0"/>
+      <c r="EN7" s="0">
+        <v>-3.3580000000000001</v>
+      </c>
       <c r="EO7" s="0">
         <v>1.883</v>
       </c>
       <c r="EP7" s="0">
         <v>-4.9370000000000003</v>
       </c>
-      <c r="EQ7" s="0"/>
-      <c r="ER7" s="0"/>
+      <c r="EQ7" s="0">
+        <v>1.635</v>
+      </c>
+      <c r="ER7" s="0">
+        <v>1.5600000000000001</v>
+      </c>
       <c r="ES7" s="0">
         <v>0.38500000000000001</v>
       </c>
-      <c r="ET7" s="0"/>
+      <c r="ET7" s="0">
+        <v>-0.81399999999999995</v>
+      </c>
       <c r="EU7" s="0">
         <v>-1.99</v>
       </c>
       <c r="EV7" s="0">
         <v>-1.3700000000000001</v>
       </c>
-      <c r="EW7" s="0"/>
+      <c r="EW7" s="0">
+        <v>-1.794</v>
+      </c>
       <c r="EX7" s="0">
         <v>-2.5739999999999998</v>
       </c>
@@ -9065,57 +9113,81 @@
       <c r="FK7" s="0">
         <v>-38.613</v>
       </c>
-      <c r="FL7" s="0"/>
+      <c r="FL7" s="0">
+        <v>30.131</v>
+      </c>
       <c r="FM7" s="0">
         <v>76.933999999999997</v>
       </c>
-      <c r="FN7" s="0"/>
+      <c r="FN7" s="0">
+        <v>37.009999999999998</v>
+      </c>
       <c r="FO7" s="0">
         <v>38.414999999999999</v>
       </c>
       <c r="FP7" s="0">
         <v>40.965000000000003</v>
       </c>
-      <c r="FQ7" s="0"/>
-      <c r="FR7" s="0"/>
+      <c r="FQ7" s="0">
+        <v>63.828000000000003</v>
+      </c>
+      <c r="FR7" s="0">
+        <v>20.693999999999999</v>
+      </c>
       <c r="FS7" s="0">
         <v>42.774000000000001</v>
       </c>
-      <c r="FT7" s="0"/>
+      <c r="FT7" s="0">
+        <v>45.981000000000002</v>
+      </c>
       <c r="FU7" s="0">
         <v>30.053999999999998</v>
       </c>
       <c r="FV7" s="0">
         <v>29.837</v>
       </c>
-      <c r="FW7" s="0"/>
+      <c r="FW7" s="0">
+        <v>33.026000000000003</v>
+      </c>
       <c r="FX7" s="0">
         <v>13.313000000000001</v>
       </c>
-      <c r="FY7" s="0"/>
+      <c r="FY7" s="0">
+        <v>61.247</v>
+      </c>
       <c r="FZ7" s="0">
         <v>84.745000000000005</v>
       </c>
-      <c r="GA7" s="0"/>
+      <c r="GA7" s="0">
+        <v>91.774000000000001</v>
+      </c>
       <c r="GB7" s="0">
         <v>40.372999999999998</v>
       </c>
       <c r="GC7" s="0">
         <v>81.939999999999998</v>
       </c>
-      <c r="GD7" s="0"/>
-      <c r="GE7" s="0"/>
+      <c r="GD7" s="0">
+        <v>61.106999999999999</v>
+      </c>
+      <c r="GE7" s="0">
+        <v>14.045999999999999</v>
+      </c>
       <c r="GF7" s="0">
         <v>24.518000000000001</v>
       </c>
-      <c r="GG7" s="0"/>
+      <c r="GG7" s="0">
+        <v>29.995999999999999</v>
+      </c>
       <c r="GH7" s="0">
         <v>92.975999999999999</v>
       </c>
       <c r="GI7" s="0">
         <v>26.93</v>
       </c>
-      <c r="GJ7" s="0"/>
+      <c r="GJ7" s="0">
+        <v>105.048</v>
+      </c>
       <c r="GK7" s="0">
         <v>57.353000000000002</v>
       </c>
@@ -9236,30 +9308,42 @@
       <c r="HX7" s="0">
         <v>80.947999999999993</v>
       </c>
-      <c r="HY7" s="0"/>
+      <c r="HY7" s="0">
+        <v>43.009</v>
+      </c>
       <c r="HZ7" s="0">
         <v>87.033000000000001</v>
       </c>
-      <c r="IA7" s="0"/>
+      <c r="IA7" s="0">
+        <v>91.959000000000003</v>
+      </c>
       <c r="IB7" s="0">
         <v>58.820999999999998</v>
       </c>
       <c r="IC7" s="0">
         <v>83.519999999999996</v>
       </c>
-      <c r="ID7" s="0"/>
-      <c r="IE7" s="0"/>
+      <c r="ID7" s="0">
+        <v>80.769000000000005</v>
+      </c>
+      <c r="IE7" s="0">
+        <v>26.925000000000001</v>
+      </c>
       <c r="IF7" s="0">
         <v>45.262</v>
       </c>
-      <c r="IG7" s="0"/>
+      <c r="IG7" s="0">
+        <v>49.752000000000002</v>
+      </c>
       <c r="IH7" s="0">
         <v>41.037999999999997</v>
       </c>
       <c r="II7" s="0">
         <v>47.109000000000002</v>
       </c>
-      <c r="IJ7" s="0"/>
+      <c r="IJ7" s="0">
+        <v>31.440000000000001</v>
+      </c>
       <c r="IK7" s="0">
         <v>23.312000000000001</v>
       </c>
@@ -9419,57 +9503,81 @@
       <c r="KK7" s="0">
         <v>18.579000000000001</v>
       </c>
-      <c r="KL7" s="0"/>
+      <c r="KL7" s="0">
+        <v>7.0350000000000001</v>
+      </c>
       <c r="KM7" s="0">
         <v>8.5429999999999993</v>
       </c>
-      <c r="KN7" s="0"/>
+      <c r="KN7" s="0">
+        <v>-6.7839999999999998</v>
+      </c>
       <c r="KO7" s="0">
         <v>-0.503</v>
       </c>
       <c r="KP7" s="0">
         <v>8.0399999999999991</v>
       </c>
-      <c r="KQ7" s="0"/>
-      <c r="KR7" s="0"/>
+      <c r="KQ7" s="0">
+        <v>-1.0049999999999999</v>
+      </c>
+      <c r="KR7" s="0">
+        <v>24.120999999999999</v>
+      </c>
       <c r="KS7" s="0">
         <v>7.2859999999999996</v>
       </c>
-      <c r="KT7" s="0"/>
+      <c r="KT7" s="0">
+        <v>4.5229999999999997</v>
+      </c>
       <c r="KU7" s="0">
         <v>12.06</v>
       </c>
       <c r="KV7" s="0">
         <v>7.0350000000000001</v>
       </c>
-      <c r="KW7" s="0"/>
+      <c r="KW7" s="0">
+        <v>12.563000000000001</v>
+      </c>
       <c r="KX7" s="0">
         <v>13.568</v>
       </c>
-      <c r="KY7" s="0"/>
+      <c r="KY7" s="0">
+        <v>34.170999999999999</v>
+      </c>
       <c r="KZ7" s="0">
         <v>51.759</v>
       </c>
-      <c r="LA7" s="0"/>
+      <c r="LA7" s="0">
+        <v>51.005000000000003</v>
+      </c>
       <c r="LB7" s="0">
         <v>18.593</v>
       </c>
       <c r="LC7" s="0">
         <v>50.250999999999998</v>
       </c>
-      <c r="LD7" s="0"/>
-      <c r="LE7" s="0"/>
+      <c r="LD7" s="0">
+        <v>-43.216000000000001</v>
+      </c>
+      <c r="LE7" s="0">
+        <v>-4.0199999999999996</v>
+      </c>
       <c r="LF7" s="0">
         <v>-4.0199999999999996</v>
       </c>
-      <c r="LG7" s="0"/>
+      <c r="LG7" s="0">
+        <v>-5.5279999999999996</v>
+      </c>
       <c r="LH7" s="0">
         <v>24.120999999999999</v>
       </c>
       <c r="LI7" s="0">
         <v>-5.5279999999999996</v>
       </c>
-      <c r="LJ7" s="0"/>
+      <c r="LJ7" s="0">
+        <v>25.628</v>
+      </c>
       <c r="LK7" s="0">
         <v>24.873999999999999</v>
       </c>
@@ -9629,30 +9737,42 @@
       <c r="NK7" s="0">
         <v>-7.9880000000000004</v>
       </c>
-      <c r="NL7" s="0"/>
+      <c r="NL7" s="0">
+        <v>6.5330000000000004</v>
+      </c>
       <c r="NM7" s="0">
         <v>0.503</v>
       </c>
-      <c r="NN7" s="0"/>
+      <c r="NN7" s="0">
+        <v>2.2610000000000001</v>
+      </c>
       <c r="NO7" s="0">
         <v>-6.5330000000000004</v>
       </c>
       <c r="NP7" s="0">
         <v>0.503</v>
       </c>
-      <c r="NQ7" s="0"/>
-      <c r="NR7" s="0"/>
+      <c r="NQ7" s="0">
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="NR7" s="0">
+        <v>22.864000000000001</v>
+      </c>
       <c r="NS7" s="0">
         <v>7.0350000000000001</v>
       </c>
-      <c r="NT7" s="0"/>
+      <c r="NT7" s="0">
+        <v>7.5380000000000003</v>
+      </c>
       <c r="NU7" s="0">
         <v>8.0399999999999991</v>
       </c>
       <c r="NV7" s="0">
         <v>7.5380000000000003</v>
       </c>
-      <c r="NW7" s="0"/>
+      <c r="NW7" s="0">
+        <v>10.050000000000001</v>
+      </c>
       <c r="NX7" s="0">
         <v>28.140999999999998</v>
       </c>
@@ -9662,112 +9782,112 @@
         <v>107</v>
       </c>
       <c r="B8" s="0">
-        <v>118.895</v>
+        <v>11.890000000000001</v>
       </c>
       <c r="C8" s="0">
-        <v>132.30500000000001</v>
+        <v>13.23</v>
       </c>
       <c r="D8" s="0">
-        <v>82.813999999999993</v>
+        <v>8.2810000000000006</v>
       </c>
       <c r="E8" s="0">
-        <v>187.636</v>
+        <v>18.763999999999999</v>
       </c>
       <c r="F8" s="0">
-        <v>151.286</v>
+        <v>15.129</v>
       </c>
       <c r="G8" s="0">
-        <v>185.70599999999999</v>
+        <v>18.571000000000002</v>
       </c>
       <c r="H8" s="0">
-        <v>226.83600000000001</v>
+        <v>22.684000000000001</v>
       </c>
       <c r="I8" s="0">
-        <v>119.70699999999999</v>
+        <v>11.971</v>
       </c>
       <c r="J8" s="0">
-        <v>94.471999999999994</v>
+        <v>9.4469999999999992</v>
       </c>
       <c r="K8" s="0">
-        <v>190.03200000000001</v>
+        <v>19.003</v>
       </c>
       <c r="L8" s="0">
-        <v>299.71899999999999</v>
+        <v>29.972000000000001</v>
       </c>
       <c r="M8" s="0">
-        <v>276.995</v>
+        <v>27.699999999999999</v>
       </c>
       <c r="N8" s="0">
-        <v>1181.1289999999999</v>
+        <v>118.113</v>
       </c>
       <c r="O8" s="0">
-        <v>1013.602</v>
+        <v>101.36</v>
       </c>
       <c r="P8" s="0">
-        <v>1143.71</v>
+        <v>114.371</v>
       </c>
       <c r="Q8" s="0">
-        <v>916.63199999999995</v>
+        <v>91.662999999999997</v>
       </c>
       <c r="R8" s="0">
-        <v>1040.2</v>
+        <v>104.02</v>
       </c>
       <c r="S8" s="0">
-        <v>972.85299999999995</v>
+        <v>97.284999999999997</v>
       </c>
       <c r="T8" s="0">
-        <v>315.96899999999999</v>
+        <v>31.597000000000001</v>
       </c>
       <c r="U8" s="0">
-        <v>229.696</v>
+        <v>22.969999999999999</v>
       </c>
       <c r="V8" s="0">
-        <v>257.45100000000002</v>
+        <v>25.745000000000001</v>
       </c>
       <c r="W8" s="0">
-        <v>151.035</v>
+        <v>15.103999999999999</v>
       </c>
       <c r="X8" s="0">
-        <v>234.72800000000001</v>
+        <v>23.472999999999999</v>
       </c>
       <c r="Y8" s="0">
-        <v>197.28899999999999</v>
+        <v>19.728999999999999</v>
       </c>
       <c r="Z8" s="0">
-        <v>257.61900000000003</v>
+        <v>25.762</v>
       </c>
       <c r="AA8" s="0">
-        <v>297.74900000000002</v>
+        <v>29.774999999999999</v>
       </c>
       <c r="AB8" s="0">
-        <v>223.08000000000001</v>
+        <v>22.308</v>
       </c>
       <c r="AC8" s="0">
-        <v>498.50900000000001</v>
+        <v>49.850999999999999</v>
       </c>
       <c r="AD8" s="0">
-        <v>208.81999999999999</v>
+        <v>20.882000000000001</v>
       </c>
       <c r="AE8" s="0">
-        <v>148.87899999999999</v>
+        <v>14.888</v>
       </c>
       <c r="AF8" s="0">
-        <v>1056.104</v>
+        <v>105.61</v>
       </c>
       <c r="AG8" s="0">
-        <v>1091.9300000000001</v>
+        <v>109.193</v>
       </c>
       <c r="AH8" s="0">
-        <v>1033.425</v>
+        <v>103.342</v>
       </c>
       <c r="AI8" s="0">
-        <v>1056.2429999999999</v>
+        <v>105.624</v>
       </c>
       <c r="AJ8" s="0">
-        <v>1016.511</v>
+        <v>101.651</v>
       </c>
       <c r="AK8" s="0">
-        <v>937.88300000000004</v>
+        <v>93.787999999999997</v>
       </c>
       <c r="AL8" s="0">
         <v>182.453</v>
@@ -10828,112 +10948,112 @@
         <v>108</v>
       </c>
       <c r="B9" s="0">
-        <v>184.65199999999999</v>
+        <v>18.465</v>
       </c>
       <c r="C9" s="0">
-        <v>198.12700000000001</v>
+        <v>19.812999999999999</v>
       </c>
       <c r="D9" s="0">
-        <v>194.292</v>
+        <v>19.428999999999998</v>
       </c>
       <c r="E9" s="0">
-        <v>182.77799999999999</v>
+        <v>18.277999999999999</v>
       </c>
       <c r="F9" s="0">
-        <v>265.447</v>
+        <v>26.545000000000002</v>
       </c>
       <c r="G9" s="0">
-        <v>224.57499999999999</v>
+        <v>22.457999999999998</v>
       </c>
       <c r="H9" s="0">
-        <v>300.03199999999998</v>
+        <v>30.003</v>
       </c>
       <c r="I9" s="0">
-        <v>340.375</v>
+        <v>34.037999999999997</v>
       </c>
       <c r="J9" s="0">
-        <v>153.32900000000001</v>
+        <v>15.333</v>
       </c>
       <c r="K9" s="0">
-        <v>227.54900000000001</v>
+        <v>22.754999999999999</v>
       </c>
       <c r="L9" s="0">
-        <v>105.095</v>
+        <v>10.509</v>
       </c>
       <c r="M9" s="0">
-        <v>100.042</v>
+        <v>10.004</v>
       </c>
       <c r="N9" s="0">
-        <v>945.952</v>
+        <v>94.594999999999999</v>
       </c>
       <c r="O9" s="0">
-        <v>592.61599999999999</v>
+        <v>59.262</v>
       </c>
       <c r="P9" s="0">
-        <v>690.73099999999999</v>
+        <v>69.072999999999993</v>
       </c>
       <c r="Q9" s="0">
-        <v>678.58900000000006</v>
+        <v>67.858999999999995</v>
       </c>
       <c r="R9" s="0">
-        <v>586.053</v>
+        <v>58.604999999999997</v>
       </c>
       <c r="S9" s="0">
-        <v>719.13300000000004</v>
+        <v>71.912999999999997</v>
       </c>
       <c r="T9" s="0">
-        <v>246.63800000000001</v>
+        <v>24.664000000000001</v>
       </c>
       <c r="U9" s="0">
-        <v>136.03999999999999</v>
+        <v>13.603999999999999</v>
       </c>
       <c r="V9" s="0">
-        <v>137.643</v>
+        <v>13.763999999999999</v>
       </c>
       <c r="W9" s="0">
-        <v>153.86799999999999</v>
+        <v>15.387</v>
       </c>
       <c r="X9" s="0">
-        <v>113.886</v>
+        <v>11.388999999999999</v>
       </c>
       <c r="Y9" s="0">
-        <v>139.761</v>
+        <v>13.976000000000001</v>
       </c>
       <c r="Z9" s="0">
-        <v>217.74000000000001</v>
+        <v>21.774000000000001</v>
       </c>
       <c r="AA9" s="0">
-        <v>254.876</v>
+        <v>25.488</v>
       </c>
       <c r="AB9" s="0">
-        <v>253.17099999999999</v>
+        <v>25.317</v>
       </c>
       <c r="AC9" s="0">
-        <v>162.58500000000001</v>
+        <v>16.257999999999999</v>
       </c>
       <c r="AD9" s="0">
-        <v>218.58099999999999</v>
+        <v>21.858000000000001</v>
       </c>
       <c r="AE9" s="0">
-        <v>252.96000000000001</v>
+        <v>25.295999999999999</v>
       </c>
       <c r="AF9" s="0">
-        <v>905.34100000000001</v>
+        <v>90.534000000000006</v>
       </c>
       <c r="AG9" s="0">
-        <v>944.96100000000001</v>
+        <v>94.495999999999995</v>
       </c>
       <c r="AH9" s="0">
-        <v>898.03300000000002</v>
+        <v>89.802999999999997</v>
       </c>
       <c r="AI9" s="0">
-        <v>796.84000000000003</v>
+        <v>79.683999999999997</v>
       </c>
       <c r="AJ9" s="0">
-        <v>857.11599999999999</v>
+        <v>85.712000000000003</v>
       </c>
       <c r="AK9" s="0">
-        <v>920.44000000000005</v>
+        <v>92.043999999999997</v>
       </c>
       <c r="AL9" s="0">
         <v>148.67500000000001</v>
@@ -11994,112 +12114,112 @@
         <v>109</v>
       </c>
       <c r="B10" s="0">
-        <v>153.58199999999999</v>
+        <v>15.358000000000001</v>
       </c>
       <c r="C10" s="0">
-        <v>95.462000000000003</v>
+        <v>9.5459999999999994</v>
       </c>
       <c r="D10" s="0">
-        <v>106.86</v>
+        <v>10.686</v>
       </c>
       <c r="E10" s="0">
-        <v>150.08199999999999</v>
+        <v>15.007999999999999</v>
       </c>
       <c r="F10" s="0">
-        <v>163.26499999999999</v>
+        <v>16.326000000000001</v>
       </c>
       <c r="G10" s="0">
-        <v>155.762</v>
+        <v>15.576000000000001</v>
       </c>
       <c r="H10" s="0">
-        <v>84.262</v>
+        <v>8.4260000000000002</v>
       </c>
       <c r="I10" s="0">
-        <v>50.454000000000001</v>
+        <v>5.0449999999999999</v>
       </c>
       <c r="J10" s="0">
-        <v>57.049999999999997</v>
+        <v>5.7050000000000001</v>
       </c>
       <c r="K10" s="0">
-        <v>83.703000000000003</v>
+        <v>8.3699999999999992</v>
       </c>
       <c r="L10" s="0">
-        <v>81.197000000000003</v>
+        <v>8.1199999999999992</v>
       </c>
       <c r="M10" s="0">
-        <v>11.699999999999999</v>
+        <v>1.1699999999999999</v>
       </c>
       <c r="N10" s="0">
-        <v>1022.218</v>
+        <v>102.22199999999999</v>
       </c>
       <c r="O10" s="0">
-        <v>1018.111</v>
+        <v>101.81100000000001</v>
       </c>
       <c r="P10" s="0">
-        <v>927.93200000000002</v>
+        <v>92.793000000000006</v>
       </c>
       <c r="Q10" s="0">
-        <v>1008.562</v>
+        <v>100.85599999999999</v>
       </c>
       <c r="R10" s="0">
-        <v>1047.702</v>
+        <v>104.77</v>
       </c>
       <c r="S10" s="0">
-        <v>964.68299999999999</v>
+        <v>96.468000000000004</v>
       </c>
       <c r="T10" s="0">
-        <v>233.61500000000001</v>
+        <v>23.361000000000001</v>
       </c>
       <c r="U10" s="0">
-        <v>229.274</v>
+        <v>22.927</v>
       </c>
       <c r="V10" s="0">
-        <v>175.631</v>
+        <v>17.562999999999999</v>
       </c>
       <c r="W10" s="0">
-        <v>210.90299999999999</v>
+        <v>21.09</v>
       </c>
       <c r="X10" s="0">
-        <v>219.43700000000001</v>
+        <v>21.943999999999999</v>
       </c>
       <c r="Y10" s="0">
-        <v>180.99600000000001</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="Z10" s="0">
-        <v>344.21300000000002</v>
+        <v>34.420999999999999</v>
       </c>
       <c r="AA10" s="0">
-        <v>368.59699999999998</v>
+        <v>36.859999999999999</v>
       </c>
       <c r="AB10" s="0">
-        <v>432.41000000000003</v>
+        <v>43.241</v>
       </c>
       <c r="AC10" s="0">
-        <v>299.12299999999999</v>
+        <v>29.911999999999999</v>
       </c>
       <c r="AD10" s="0">
-        <v>323.22000000000003</v>
+        <v>32.322000000000003</v>
       </c>
       <c r="AE10" s="0">
-        <v>342.48700000000002</v>
+        <v>34.249000000000002</v>
       </c>
       <c r="AF10" s="0">
-        <v>1102.6600000000001</v>
+        <v>110.26600000000001</v>
       </c>
       <c r="AG10" s="0">
-        <v>1147.335</v>
+        <v>114.733</v>
       </c>
       <c r="AH10" s="0">
-        <v>1231.9390000000001</v>
+        <v>123.194</v>
       </c>
       <c r="AI10" s="0">
-        <v>1107.903</v>
+        <v>110.79000000000001</v>
       </c>
       <c r="AJ10" s="0">
-        <v>1147.451</v>
+        <v>114.745</v>
       </c>
       <c r="AK10" s="0">
-        <v>1191.7670000000001</v>
+        <v>119.17700000000001</v>
       </c>
       <c r="AL10" s="0">
         <v>168.53</v>

</xml_diff>